<commit_message>
Replace location menu templates with client CSV data unchanged
Convert shilpa_enterprise_menu_1401.csv to the standard 11-column xlsx format
and copy byte-identically to all three location template filenames. Keep the
CSV as the canonical source for scripts/generate_location_menus.py.

Co-authored-by: Vigneshwari116 <Vigneshwari116@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assets/templates/Shilpa_Enterprise_menu_items_CLIENT_FINAL.xlsx
+++ b/assets/templates/Shilpa_Enterprise_menu_items_CLIENT_FINAL.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Menu" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K47"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -499,7 +499,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>24</t>
@@ -510,8 +509,6 @@
           <t>pc</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>10</t>
@@ -544,7 +541,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>24</t>
@@ -555,8 +551,6 @@
           <t>pc</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr">
         <is>
           <t>15</t>
@@ -589,7 +583,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>24</t>
@@ -600,8 +593,6 @@
           <t>pc</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr">
         <is>
           <t>20</t>
@@ -634,7 +625,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>20</t>
@@ -650,7 +640,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr">
         <is>
           <t>60</t>
@@ -683,7 +672,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>5</t>
@@ -699,7 +687,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
           <t>110</t>
@@ -732,7 +719,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>14</t>
@@ -748,7 +734,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr">
         <is>
           <t>90</t>
@@ -758,7 +743,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BURGERS</t>
+          <t xml:space="preserve">BURGERS </t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -781,7 +766,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>13</t>
@@ -797,7 +781,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr">
         <is>
           <t>95</t>
@@ -807,7 +790,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BURGERS</t>
+          <t xml:space="preserve">BURGERS </t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -830,7 +813,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>13</t>
@@ -846,7 +828,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr">
         <is>
           <t>100</t>
@@ -856,7 +837,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BURGERS</t>
+          <t xml:space="preserve">BURGERS </t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -879,7 +860,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>13</t>
@@ -895,7 +875,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr">
         <is>
           <t>65</t>
@@ -905,7 +884,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BURGERS</t>
+          <t xml:space="preserve">BURGERS </t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -928,7 +907,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>10</t>
@@ -939,8 +917,6 @@
           <t>pc</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr">
         <is>
           <t>129</t>
@@ -973,7 +949,6 @@
           <t>8</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>40</t>
@@ -984,8 +959,6 @@
           <t>pc</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr">
         <is>
           <t>109</t>
@@ -1018,7 +991,6 @@
           <t>2</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>10</t>
@@ -1029,8 +1001,6 @@
           <t>pc</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
           <t>99</t>
@@ -1058,8 +1028,11 @@
           <t>FRIED ITEM</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
           <t>4</t>
@@ -1070,8 +1043,6 @@
           <t>pc</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
           <t>119</t>
@@ -1091,7 +1062,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Thai Crispy</t>
+          <t>Thai Crispy.m</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1104,7 +1075,6 @@
           <t>5</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>10</t>
@@ -1115,8 +1085,6 @@
           <t>pc</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
           <t>385</t>
@@ -1136,7 +1104,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Thai Crispy</t>
+          <t>Thai Crispy.l</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1149,7 +1117,6 @@
           <t>10</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>10</t>
@@ -1160,8 +1127,6 @@
           <t>pc</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr">
         <is>
           <t>765</t>
@@ -1171,7 +1136,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>FRIED ITEMS</t>
+          <t xml:space="preserve">FRIED ITEMS </t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1181,7 +1146,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Chicken Popcorn Small</t>
+          <t>Chicken Popcorn</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1191,11 +1156,14 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
+          <t>550</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
           <t>80</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>g</t>
@@ -1206,7 +1174,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr">
         <is>
           <t>70</t>
@@ -1216,7 +1183,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>FRIED ITEMS</t>
+          <t xml:space="preserve">FRIED ITEMS </t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1239,7 +1206,6 @@
           <t>3</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>27</t>
@@ -1255,7 +1221,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr">
         <is>
           <t>99</t>
@@ -1265,7 +1230,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>FRIED ITEMS</t>
+          <t xml:space="preserve">FRIED ITEMS </t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1288,7 +1253,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
       <c r="G19" t="inlineStr">
         <is>
           <t>10</t>
@@ -1304,7 +1268,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
           <t>80</t>
@@ -1314,7 +1277,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>FRIED ITEMS</t>
+          <t xml:space="preserve">FRIED ITEMS </t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1337,7 +1300,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
           <t>10</t>
@@ -1348,9 +1310,7 @@
           <t>pc</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr">
+      <c r="I20" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -1359,7 +1319,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>FRIED ITEMS</t>
+          <t xml:space="preserve">FRIED ITEMS </t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1382,8 +1342,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1394,7 +1352,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr">
         <is>
           <t>90</t>
@@ -1404,7 +1361,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>FRIED ITEMS</t>
+          <t xml:space="preserve">FRIED ITEMS </t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1427,8 +1384,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1439,7 +1394,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr">
         <is>
           <t>99</t>
@@ -1449,7 +1403,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FRIED ITEMS</t>
+          <t xml:space="preserve">FRIED ITEMS </t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1472,7 +1426,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
       <c r="G23" t="inlineStr">
         <is>
           <t>10</t>
@@ -1488,7 +1441,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr">
         <is>
           <t>80</t>
@@ -1521,7 +1473,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
       <c r="G24" t="inlineStr">
         <is>
           <t>4</t>
@@ -1537,7 +1488,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr">
         <is>
           <t>85</t>
@@ -1570,7 +1520,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
           <t>14</t>
@@ -1586,7 +1535,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr">
         <is>
           <t>90</t>
@@ -1614,25 +1562,6 @@
           <t>COMBO</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1655,25 +1584,6 @@
           <t>COMBO</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1701,8 +1611,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1713,8 +1621,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1742,8 +1648,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1754,13 +1658,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SAUCES</t>
+          <t xml:space="preserve">SAUCES </t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1783,8 +1685,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1795,13 +1695,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SAUCES</t>
+          <t xml:space="preserve">SAUCES </t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1824,8 +1722,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1836,13 +1732,11 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SAUCES</t>
+          <t xml:space="preserve">SAUCES </t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1865,8 +1759,6 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>pc</t>
@@ -1877,28 +1769,26 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SAUCES</t>
+          <t>SNACKS</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>PACKING COVER</t>
+          <t>French Fries</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PACKING COVER</t>
+          <t>French Fries</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>SAUCE/DRY STOCK</t>
+          <t>SNACKS</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1906,11 +1796,14 @@
           <t>1</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>pc</t>
+          <t>g</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -1918,81 +1811,68 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SAUCES</t>
+          <t>SNACKS</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>SNACK BOX</t>
+          <t>CHICKEN STRIPS</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>SNACK BOX</t>
+          <t>CHICKEN STRIPS</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>SAUCE/DRY STOCK</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
+          <t>COMBO</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t xml:space="preserve">SNACKS </t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Chicken 65</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Chicken 65</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
           <t>SNACKS</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>French Fries</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>French Fries Small</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>SNACKS</t>
-        </is>
-      </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>80</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pc</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2000,40 +1880,38 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J35" t="inlineStr"/>
       <c r="K35" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>85</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t xml:space="preserve">SNACKS </t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Chicken Cheese Shotz</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Chicken Cheese Shotz</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
           <t>SNACKS</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>CHICKEN STRIPS</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>CHICKEN STRIPS</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>COMBO</t>
-        </is>
-      </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr"/>
+          <t>6</t>
+        </is>
+      </c>
       <c r="G36" t="inlineStr">
         <is>
           <t>50</t>
@@ -2049,41 +1927,43 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>90</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t xml:space="preserve">SNACKS </t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Chicken Fingers</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Chicken Fingers</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
           <t>SNACKS</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Chicken 65</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>Chicken 65</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>SNACKS</t>
-        </is>
-      </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="H37" t="inlineStr">
         <is>
           <t>pc</t>
@@ -2094,43 +1974,41 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>60</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t xml:space="preserve">SNACKS </t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Chicken Momos</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Chicken Momos</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
           <t>SNACKS</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Chicken Cheese Shotz</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>Chicken Cheese Shotz</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>SNACKS</t>
-        </is>
-      </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr"/>
+          <t>4</t>
+        </is>
+      </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>40</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2141,45 +2019,38 @@
       <c r="I38" t="inlineStr">
         <is>
           <t>0</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr"/>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>90</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t xml:space="preserve">SNACKS </t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Chicken Nuggets</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Chicken Nuggets</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
           <t>SNACKS</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Chicken Fingers</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>Chicken Fingers</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>SNACKS</t>
-        </is>
-      </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
+          <t>4</t>
+        </is>
+      </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>60</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2192,43 +2063,41 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>55</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t xml:space="preserve">SNACKS </t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Pizza Pocket</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Pizza Pocket</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
           <t>SNACKS</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Chicken Momos</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>Chicken Momos</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>SNACKS</t>
-        </is>
-      </c>
       <c r="E40" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr"/>
       <c r="G40" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>28</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2241,39 +2110,41 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t xml:space="preserve">SNACKS </t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Veg Finger</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Veg Finger</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
           <t>SNACKS</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Chicken Nuggets</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>Chicken Nuggets</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>SNACKS</t>
-        </is>
-      </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr"/>
+          <t>3</t>
+        </is>
+      </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>33</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2286,7 +2157,6 @@
           <t>0</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr">
         <is>
           <t>55</t>
@@ -2296,281 +2166,235 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t xml:space="preserve">SNACKS </t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>chicken popcorn large</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Chicken Popcorn</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
           <t>SNACKS</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Pizza Pocket</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>Pizza Pocket</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>SNACKS</t>
-        </is>
-      </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr"/>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>gms</t>
+        </is>
+      </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>120</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>pc</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr"/>
+          <t>g</t>
+        </is>
+      </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>120</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t xml:space="preserve">SNACKS </t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>masala fries Large</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>French Fries</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
           <t>SNACKS</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Veg Finger</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Veg Finger</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>SNACKS</t>
-        </is>
-      </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr"/>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>gms</t>
+        </is>
+      </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>120</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>pc</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr"/>
+          <t>g</t>
+        </is>
+      </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>99</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SNACKS</t>
+          <t>STOCK</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>chicken popcorn large</t>
+          <t>Burger Bun With Sesame</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Chicken Popcorn Large</t>
+          <t>Burger Bun With Sesame</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>SNACKS</t>
+          <t>STOCK</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>120</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pc</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
           <t>0</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr"/>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>120</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SNACKS</t>
+          <t>STOCK</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>masala fries Large</t>
+          <t>Paratha</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>French Fries Large</t>
+          <t>Paratha</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>SNACKS</t>
+          <t>STOCK</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>120</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>pc</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
           <t>0</t>
-        </is>
-      </c>
-      <c r="J45" t="inlineStr"/>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>99</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>STOCK</t>
+          <t>SAUCES</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Burger Bun With Sesame</t>
+          <t>PACKING COVER</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Bun</t>
+          <t>PACKING COVER</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>STOCK</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr"/>
-      <c r="K46" t="inlineStr"/>
+          <t>SAUCE/DRY STOCK</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>STOCK</t>
+          <t>SAUCES</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Paratha</t>
+          <t>SNACK BOX</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Paratha</t>
+          <t>SNACK BOX</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>STOCK</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>pc</t>
-        </is>
-      </c>
-      <c r="I47" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J47" t="inlineStr"/>
-      <c r="K47" t="inlineStr"/>
-    </row>
+          <t>SAUCE/DRY STOCK</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>SAUCES</t>
+        </is>
+      </c>
+    </row>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>